<commit_message>
add exit plan to daily stock report
</commit_message>
<xml_diff>
--- a/A股每日选股报告页面设计/public/reports/20260624/stock_pick_20260624.xlsx
+++ b/A股每日选股报告页面设计/public/reports/20260624/stock_pick_20260624.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="准确性评估" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'选股详情'!$A$1:$Z$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'选股详情'!$A$1:$AG$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'技术诊断'!$A$3:$F$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'筛选漏斗'!$A$3:$E$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'准确性评估'!$A$9:$G$32</definedName>
@@ -491,9 +491,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StockPicks" displayName="StockPicks" ref="A1:Z21" headerRowCount="1">
-  <autoFilter ref="A1:Z21"/>
-  <tableColumns count="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StockPicks" displayName="StockPicks" ref="A1:AG21" headerRowCount="1">
+  <autoFilter ref="A1:AG21"/>
+  <tableColumns count="33">
     <tableColumn id="1" name="排名"/>
     <tableColumn id="2" name="代码"/>
     <tableColumn id="3" name="名称"/>
@@ -520,6 +520,13 @@
     <tableColumn id="24" name="板块排名分位"/>
     <tableColumn id="25" name="板块内排名分位"/>
     <tableColumn id="26" name="入场时机"/>
+    <tableColumn id="27" name="计划持有日"/>
+    <tableColumn id="28" name="止损价"/>
+    <tableColumn id="29" name="第一止盈"/>
+    <tableColumn id="30" name="第二止盈"/>
+    <tableColumn id="31" name="移动止盈"/>
+    <tableColumn id="32" name="盈亏比"/>
+    <tableColumn id="33" name="退出计划"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -874,7 +881,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>智微智能(1339)</t>
+          <t>智微智能(001339)</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr"/>
@@ -1059,7 +1066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z21"/>
+  <dimension ref="A1:AG21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1088,6 +1095,13 @@
     <col width="8" customWidth="1" min="24" max="24"/>
     <col width="9" customWidth="1" min="25" max="25"/>
     <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="8" customWidth="1" min="27" max="27"/>
+    <col width="8" customWidth="1" min="28" max="28"/>
+    <col width="8" customWidth="1" min="29" max="29"/>
+    <col width="8" customWidth="1" min="30" max="30"/>
+    <col width="8" customWidth="1" min="31" max="31"/>
+    <col width="8" customWidth="1" min="32" max="32"/>
+    <col width="28" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1221,13 +1235,50 @@
           <t>入场时机</t>
         </is>
       </c>
+      <c r="AA1" s="7" t="inlineStr">
+        <is>
+          <t>计划持有日</t>
+        </is>
+      </c>
+      <c r="AB1" s="7" t="inlineStr">
+        <is>
+          <t>止损价</t>
+        </is>
+      </c>
+      <c r="AC1" s="7" t="inlineStr">
+        <is>
+          <t>第一止盈</t>
+        </is>
+      </c>
+      <c r="AD1" s="7" t="inlineStr">
+        <is>
+          <t>第二止盈</t>
+        </is>
+      </c>
+      <c r="AE1" s="7" t="inlineStr">
+        <is>
+          <t>移动止盈</t>
+        </is>
+      </c>
+      <c r="AF1" s="7" t="inlineStr">
+        <is>
+          <t>盈亏比</t>
+        </is>
+      </c>
+      <c r="AG1" s="7" t="inlineStr">
+        <is>
+          <t>退出计划</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="n">
-        <v>1339</v>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>001339</t>
+        </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
@@ -1303,6 +1354,29 @@
       <c r="Z2" s="4" t="inlineStr">
         <is>
           <t>🟡 首日上涨，可关注</t>
+        </is>
+      </c>
+      <c r="AA2" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB2" s="4" t="n">
+        <v>127.36</v>
+      </c>
+      <c r="AC2" s="4" t="n">
+        <v>152.29</v>
+      </c>
+      <c r="AD2" s="4" t="n">
+        <v>161.87</v>
+      </c>
+      <c r="AE2" s="4" t="n">
+        <v>128.67</v>
+      </c>
+      <c r="AF2" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AG2" s="4" t="inlineStr">
+        <is>
+          <t>3日计划；跌破127.36止损；上冲152.29先止盈；破MA5/移动止盈128.67减仓</t>
         </is>
       </c>
     </row>
@@ -1310,8 +1384,10 @@
       <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="n">
-        <v>823</v>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>000823</t>
+        </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
@@ -1387,6 +1463,29 @@
       <c r="Z3" s="4" t="inlineStr">
         <is>
           <t>🟡 首日上涨，可关注</t>
+        </is>
+      </c>
+      <c r="AA3" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB3" s="4" t="n">
+        <v>21.87</v>
+      </c>
+      <c r="AC3" s="4" t="n">
+        <v>26.41</v>
+      </c>
+      <c r="AD3" s="4" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="AE3" s="4" t="n">
+        <v>22.02</v>
+      </c>
+      <c r="AF3" s="4" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="AG3" s="4" t="inlineStr">
+        <is>
+          <t>3日计划；跌破21.87止损；上冲26.41先止盈；破MA5/移动止盈22.02减仓</t>
         </is>
       </c>
     </row>
@@ -1394,8 +1493,10 @@
       <c r="A4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="n">
-        <v>603938</v>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>603938</t>
+        </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
@@ -1471,6 +1572,29 @@
       <c r="Z4" s="4" t="inlineStr">
         <is>
           <t>🟠 连涨多日，等回调再入</t>
+        </is>
+      </c>
+      <c r="AA4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB4" s="4" t="n">
+        <v>66.62</v>
+      </c>
+      <c r="AC4" s="4" t="n">
+        <v>79.90000000000001</v>
+      </c>
+      <c r="AD4" s="4" t="n">
+        <v>88.17</v>
+      </c>
+      <c r="AE4" s="4" t="n">
+        <v>66.62</v>
+      </c>
+      <c r="AF4" s="4" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="AG4" s="4" t="inlineStr">
+        <is>
+          <t>3日计划；跌破66.62止损；上冲79.90先止盈；破MA5/移动止盈66.62减仓</t>
         </is>
       </c>
     </row>
@@ -1478,8 +1602,10 @@
       <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="n">
-        <v>603713</v>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>603713</t>
+        </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
@@ -1555,6 +1681,29 @@
       <c r="Z5" s="4" t="inlineStr">
         <is>
           <t>🟠 连涨多日，等回调再入</t>
+        </is>
+      </c>
+      <c r="AA5" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB5" s="4" t="n">
+        <v>63.96</v>
+      </c>
+      <c r="AC5" s="4" t="n">
+        <v>76.47</v>
+      </c>
+      <c r="AD5" s="4" t="n">
+        <v>81.29000000000001</v>
+      </c>
+      <c r="AE5" s="4" t="n">
+        <v>64.56</v>
+      </c>
+      <c r="AF5" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AG5" s="4" t="inlineStr">
+        <is>
+          <t>3日计划；跌破63.96止损；上冲76.47先止盈；破MA5/移动止盈64.56减仓</t>
         </is>
       </c>
     </row>
@@ -1562,8 +1711,10 @@
       <c r="A6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="n">
-        <v>672</v>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>000672</t>
+        </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
@@ -1639,6 +1790,29 @@
       <c r="Z6" s="4" t="inlineStr">
         <is>
           <t>🟠 连涨多日，等回调再入</t>
+        </is>
+      </c>
+      <c r="AA6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB6" s="4" t="n">
+        <v>20.04</v>
+      </c>
+      <c r="AC6" s="4" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AD6" s="4" t="n">
+        <v>25.47</v>
+      </c>
+      <c r="AE6" s="4" t="n">
+        <v>20.14</v>
+      </c>
+      <c r="AF6" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AG6" s="4" t="inlineStr">
+        <is>
+          <t>3日计划；跌破20.04止损；上冲23.96先止盈；破MA5/移动止盈20.14减仓</t>
         </is>
       </c>
     </row>
@@ -1646,8 +1820,10 @@
       <c r="A7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="n">
-        <v>50</v>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>000050</t>
+        </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
@@ -1723,6 +1899,29 @@
       <c r="Z7" s="4" t="inlineStr">
         <is>
           <t>🟠 连涨多日，等回调再入</t>
+        </is>
+      </c>
+      <c r="AA7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB7" s="4" t="n">
+        <v>9.970000000000001</v>
+      </c>
+      <c r="AC7" s="4" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="AD7" s="4" t="n">
+        <v>12.77</v>
+      </c>
+      <c r="AE7" s="4" t="n">
+        <v>9.970000000000001</v>
+      </c>
+      <c r="AF7" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AG7" s="4" t="inlineStr">
+        <is>
+          <t>3日计划；跌破9.97止损；上冲11.92先止盈；破MA5/移动止盈9.97减仓</t>
         </is>
       </c>
     </row>
@@ -1730,8 +1929,10 @@
       <c r="A8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="n">
-        <v>603005</v>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>603005</t>
+        </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -1807,6 +2008,29 @@
       <c r="Z8" s="4" t="inlineStr">
         <is>
           <t>🟠 连涨多日，等回调再入</t>
+        </is>
+      </c>
+      <c r="AA8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB8" s="4" t="n">
+        <v>46.16</v>
+      </c>
+      <c r="AC8" s="4" t="n">
+        <v>55.23</v>
+      </c>
+      <c r="AD8" s="4" t="n">
+        <v>60.82</v>
+      </c>
+      <c r="AE8" s="4" t="n">
+        <v>46.16</v>
+      </c>
+      <c r="AF8" s="4" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="AG8" s="4" t="inlineStr">
+        <is>
+          <t>3日计划；跌破46.16止损；上冲55.23先止盈；破MA5/移动止盈46.16减仓</t>
         </is>
       </c>
     </row>
@@ -1814,8 +2038,10 @@
       <c r="A9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="n">
-        <v>600552</v>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>600552</t>
+        </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
@@ -1891,6 +2117,29 @@
       <c r="Z9" s="4" t="inlineStr">
         <is>
           <t>🟠 远离均线，不宜追高</t>
+        </is>
+      </c>
+      <c r="AA9" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB9" s="4" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="AC9" s="4" t="n">
+        <v>31.22</v>
+      </c>
+      <c r="AD9" s="4" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="AE9" s="4" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="AF9" s="4" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="AG9" s="4" t="inlineStr">
+        <is>
+          <t>3日计划；跌破25.90止损；上冲31.22先止盈；破MA5/移动止盈25.90减仓</t>
         </is>
       </c>
     </row>
@@ -1898,8 +2147,10 @@
       <c r="A10" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="4" t="n">
-        <v>691</v>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>000691</t>
+        </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
@@ -1975,6 +2226,29 @@
       <c r="Z10" s="4" t="inlineStr">
         <is>
           <t>🟠 远离均线，不宜追高</t>
+        </is>
+      </c>
+      <c r="AA10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB10" s="4" t="n">
+        <v>12.55</v>
+      </c>
+      <c r="AC10" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD10" s="4" t="n">
+        <v>15.97</v>
+      </c>
+      <c r="AE10" s="4" t="n">
+        <v>12.55</v>
+      </c>
+      <c r="AF10" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AG10" s="4" t="inlineStr">
+        <is>
+          <t>3日计划；跌破12.55止损；上冲15.00先止盈；破MA5/移动止盈12.55减仓</t>
         </is>
       </c>
     </row>
@@ -1982,8 +2256,10 @@
       <c r="A11" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="4" t="n">
-        <v>600563</v>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>600563</t>
+        </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
@@ -2059,6 +2335,29 @@
       <c r="Z11" s="4" t="inlineStr">
         <is>
           <t>🟡 首日上涨，可关注</t>
+        </is>
+      </c>
+      <c r="AA11" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB11" s="4" t="n">
+        <v>166.25</v>
+      </c>
+      <c r="AC11" s="4" t="n">
+        <v>198.78</v>
+      </c>
+      <c r="AD11" s="4" t="n">
+        <v>216.99</v>
+      </c>
+      <c r="AE11" s="4" t="n">
+        <v>167.08</v>
+      </c>
+      <c r="AF11" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AG11" s="4" t="inlineStr">
+        <is>
+          <t>5日计划；跌破166.25止损；上冲198.78先止盈；破MA5/移动止盈167.08减仓</t>
         </is>
       </c>
     </row>
@@ -2066,8 +2365,10 @@
       <c r="A12" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="4" t="n">
-        <v>603127</v>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>603127</t>
+        </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
@@ -2143,6 +2444,29 @@
       <c r="Z12" s="4" t="inlineStr">
         <is>
           <t>🟡 首日上涨，可关注</t>
+        </is>
+      </c>
+      <c r="AA12" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB12" s="4" t="n">
+        <v>35.41</v>
+      </c>
+      <c r="AC12" s="4" t="n">
+        <v>42.34</v>
+      </c>
+      <c r="AD12" s="4" t="n">
+        <v>45.01</v>
+      </c>
+      <c r="AE12" s="4" t="n">
+        <v>36.04</v>
+      </c>
+      <c r="AF12" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AG12" s="4" t="inlineStr">
+        <is>
+          <t>5日计划；跌破35.41止损；上冲42.34先止盈；破MA5/移动止盈36.04减仓</t>
         </is>
       </c>
     </row>
@@ -2150,8 +2474,10 @@
       <c r="A13" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="4" t="n">
-        <v>603757</v>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>603757</t>
+        </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
@@ -2227,6 +2553,29 @@
       <c r="Z13" s="4" t="inlineStr">
         <is>
           <t>🟠 连涨多日，等回调再入</t>
+        </is>
+      </c>
+      <c r="AA13" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB13" s="4" t="n">
+        <v>68.54000000000001</v>
+      </c>
+      <c r="AC13" s="4" t="n">
+        <v>81.95</v>
+      </c>
+      <c r="AD13" s="4" t="n">
+        <v>87.43000000000001</v>
+      </c>
+      <c r="AE13" s="4" t="n">
+        <v>68.54000000000001</v>
+      </c>
+      <c r="AF13" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AG13" s="4" t="inlineStr">
+        <is>
+          <t>3日计划；跌破68.54止损；上冲81.95先止盈；破MA5/移动止盈68.54减仓</t>
         </is>
       </c>
     </row>
@@ -2234,8 +2583,10 @@
       <c r="A14" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="4" t="n">
-        <v>603259</v>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>603259</t>
+        </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
@@ -2311,6 +2662,29 @@
       <c r="Z14" s="4" t="inlineStr">
         <is>
           <t>🟠 远离均线，不宜追高</t>
+        </is>
+      </c>
+      <c r="AA14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB14" s="4" t="n">
+        <v>107.52</v>
+      </c>
+      <c r="AC14" s="4" t="n">
+        <v>128.01</v>
+      </c>
+      <c r="AD14" s="4" t="n">
+        <v>135.89</v>
+      </c>
+      <c r="AE14" s="4" t="n">
+        <v>110.15</v>
+      </c>
+      <c r="AF14" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AG14" s="4" t="inlineStr">
+        <is>
+          <t>3日计划；跌破107.52止损；上冲128.01先止盈；破MA5/移动止盈110.15减仓</t>
         </is>
       </c>
     </row>
@@ -2318,8 +2692,10 @@
       <c r="A15" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="4" t="n">
-        <v>925</v>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>000925</t>
+        </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
@@ -2395,6 +2771,29 @@
       <c r="Z15" s="4" t="inlineStr">
         <is>
           <t>🟡 首日上涨，可关注</t>
+        </is>
+      </c>
+      <c r="AA15" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB15" s="4" t="n">
+        <v>8.449999999999999</v>
+      </c>
+      <c r="AC15" s="4" t="n">
+        <v>10.11</v>
+      </c>
+      <c r="AD15" s="4" t="n">
+        <v>10.74</v>
+      </c>
+      <c r="AE15" s="4" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="AF15" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AG15" s="4" t="inlineStr">
+        <is>
+          <t>5日计划；跌破8.45止损；上冲10.11先止盈；破MA5/移动止盈8.50减仓</t>
         </is>
       </c>
     </row>
@@ -2402,8 +2801,10 @@
       <c r="A16" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="4" t="n">
-        <v>600497</v>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>600497</t>
+        </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
@@ -2479,6 +2880,29 @@
       <c r="Z16" s="4" t="inlineStr">
         <is>
           <t>🟠 远离均线，不宜追高</t>
+        </is>
+      </c>
+      <c r="AA16" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB16" s="4" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="AC16" s="4" t="n">
+        <v>13.46</v>
+      </c>
+      <c r="AD16" s="4" t="n">
+        <v>14.33</v>
+      </c>
+      <c r="AE16" s="4" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="AF16" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AG16" s="4" t="inlineStr">
+        <is>
+          <t>3日计划；跌破11.25止损；上冲13.46先止盈；破MA5/移动止盈11.25减仓</t>
         </is>
       </c>
     </row>
@@ -2486,8 +2910,10 @@
       <c r="A17" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="4" t="n">
-        <v>600096</v>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>600096</t>
+        </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
@@ -2563,6 +2989,29 @@
       <c r="Z17" s="4" t="inlineStr">
         <is>
           <t>🟡 首日上涨，可关注</t>
+        </is>
+      </c>
+      <c r="AA17" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB17" s="4" t="n">
+        <v>31.73</v>
+      </c>
+      <c r="AC17" s="4" t="n">
+        <v>37.94</v>
+      </c>
+      <c r="AD17" s="4" t="n">
+        <v>40.33</v>
+      </c>
+      <c r="AE17" s="4" t="n">
+        <v>32.23</v>
+      </c>
+      <c r="AF17" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AG17" s="4" t="inlineStr">
+        <is>
+          <t>5日计划；跌破31.73止损；上冲37.94先止盈；破MA5/移动止盈32.23减仓</t>
         </is>
       </c>
     </row>
@@ -2570,8 +3019,10 @@
       <c r="A18" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="4" t="n">
-        <v>603281</v>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>603281</t>
+        </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
@@ -2647,6 +3098,29 @@
       <c r="Z18" s="4" t="inlineStr">
         <is>
           <t>🟠 连涨2天，注意节奏</t>
+        </is>
+      </c>
+      <c r="AA18" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB18" s="4" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="AC18" s="4" t="n">
+        <v>45.19</v>
+      </c>
+      <c r="AD18" s="4" t="n">
+        <v>48.04</v>
+      </c>
+      <c r="AE18" s="4" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="AF18" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AG18" s="4" t="inlineStr">
+        <is>
+          <t>5日计划；跌破37.80止损；上冲45.19先止盈；破MA5/移动止盈38.30减仓</t>
         </is>
       </c>
     </row>
@@ -2654,8 +3128,10 @@
       <c r="A19" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="4" t="n">
-        <v>960</v>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>000960</t>
+        </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
@@ -2731,6 +3207,29 @@
       <c r="Z19" s="4" t="inlineStr">
         <is>
           <t>🟡 首日上涨，可关注</t>
+        </is>
+      </c>
+      <c r="AA19" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB19" s="4" t="n">
+        <v>43.34</v>
+      </c>
+      <c r="AC19" s="4" t="n">
+        <v>51.82</v>
+      </c>
+      <c r="AD19" s="4" t="n">
+        <v>56.31</v>
+      </c>
+      <c r="AE19" s="4" t="n">
+        <v>43.34</v>
+      </c>
+      <c r="AF19" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AG19" s="4" t="inlineStr">
+        <is>
+          <t>3日计划；跌破43.34止损；上冲51.82先止盈；破MA5/移动止盈43.34减仓</t>
         </is>
       </c>
     </row>
@@ -2738,8 +3237,10 @@
       <c r="A20" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="4" t="n">
-        <v>605111</v>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>605111</t>
+        </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
@@ -2815,6 +3316,29 @@
       <c r="Z20" s="4" t="inlineStr">
         <is>
           <t>🟢 回调即机会</t>
+        </is>
+      </c>
+      <c r="AA20" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB20" s="4" t="n">
+        <v>73.93000000000001</v>
+      </c>
+      <c r="AC20" s="4" t="n">
+        <v>88.39</v>
+      </c>
+      <c r="AD20" s="4" t="n">
+        <v>94.56</v>
+      </c>
+      <c r="AE20" s="4" t="n">
+        <v>74.37</v>
+      </c>
+      <c r="AF20" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AG20" s="4" t="inlineStr">
+        <is>
+          <t>3日计划；跌破73.93止损；上冲88.39先止盈；破MA5/移动止盈74.37减仓</t>
         </is>
       </c>
     </row>
@@ -2822,8 +3346,10 @@
       <c r="A21" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="4" t="n">
-        <v>603976</v>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>603976</t>
+        </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
@@ -2901,9 +3427,32 @@
           <t>🟡 首日上涨，可关注</t>
         </is>
       </c>
+      <c r="AA21" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB21" s="4" t="n">
+        <v>27.14</v>
+      </c>
+      <c r="AC21" s="4" t="n">
+        <v>32.45</v>
+      </c>
+      <c r="AD21" s="4" t="n">
+        <v>35.46</v>
+      </c>
+      <c r="AE21" s="4" t="n">
+        <v>27.16</v>
+      </c>
+      <c r="AF21" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AG21" s="4" t="inlineStr">
+        <is>
+          <t>3日计划；跌破27.14止损；上冲32.45先止盈；破MA5/移动止盈27.16减仓</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z21"/>
+  <autoFilter ref="A1:AG21"/>
   <conditionalFormatting sqref="G2:G21">
     <cfRule type="colorScale" priority="1">
       <colorScale>

</xml_diff>

<commit_message>
add short term exit plans
</commit_message>
<xml_diff>
--- a/A股每日选股报告页面设计/public/reports/20260624/stock_pick_20260624.xlsx
+++ b/A股每日选股报告页面设计/public/reports/20260624/stock_pick_20260624.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="准确性评估" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'选股详情'!$A$1:$AG$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'选股详情'!$A$1:$AP$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'技术诊断'!$A$3:$F$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'筛选漏斗'!$A$3:$E$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'准确性评估'!$A$9:$G$32</definedName>
@@ -491,9 +491,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StockPicks" displayName="StockPicks" ref="A1:AG21" headerRowCount="1">
-  <autoFilter ref="A1:AG21"/>
-  <tableColumns count="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StockPicks" displayName="StockPicks" ref="A1:AP21" headerRowCount="1">
+  <autoFilter ref="A1:AP21"/>
+  <tableColumns count="42">
     <tableColumn id="1" name="排名"/>
     <tableColumn id="2" name="代码"/>
     <tableColumn id="3" name="名称"/>
@@ -527,6 +527,15 @@
     <tableColumn id="31" name="移动止盈"/>
     <tableColumn id="32" name="盈亏比"/>
     <tableColumn id="33" name="退出计划"/>
+    <tableColumn id="34" name="第1日止损"/>
+    <tableColumn id="35" name="第1日止盈"/>
+    <tableColumn id="36" name="第1日计划"/>
+    <tableColumn id="37" name="第2日止损"/>
+    <tableColumn id="38" name="第2日止盈"/>
+    <tableColumn id="39" name="第2日计划"/>
+    <tableColumn id="40" name="第3日止损"/>
+    <tableColumn id="41" name="第3日止盈"/>
+    <tableColumn id="42" name="第3日计划"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1066,7 +1075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG21"/>
+  <dimension ref="A1:AP21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1102,6 +1111,15 @@
     <col width="8" customWidth="1" min="31" max="31"/>
     <col width="8" customWidth="1" min="32" max="32"/>
     <col width="28" customWidth="1" min="33" max="33"/>
+    <col width="8" customWidth="1" min="34" max="34"/>
+    <col width="8" customWidth="1" min="35" max="35"/>
+    <col width="28" customWidth="1" min="36" max="36"/>
+    <col width="8" customWidth="1" min="37" max="37"/>
+    <col width="8" customWidth="1" min="38" max="38"/>
+    <col width="28" customWidth="1" min="39" max="39"/>
+    <col width="8" customWidth="1" min="40" max="40"/>
+    <col width="8" customWidth="1" min="41" max="41"/>
+    <col width="28" customWidth="1" min="42" max="42"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1270,6 +1288,51 @@
           <t>退出计划</t>
         </is>
       </c>
+      <c r="AH1" s="7" t="inlineStr">
+        <is>
+          <t>第1日止损</t>
+        </is>
+      </c>
+      <c r="AI1" s="7" t="inlineStr">
+        <is>
+          <t>第1日止盈</t>
+        </is>
+      </c>
+      <c r="AJ1" s="7" t="inlineStr">
+        <is>
+          <t>第1日计划</t>
+        </is>
+      </c>
+      <c r="AK1" s="7" t="inlineStr">
+        <is>
+          <t>第2日止损</t>
+        </is>
+      </c>
+      <c r="AL1" s="7" t="inlineStr">
+        <is>
+          <t>第2日止盈</t>
+        </is>
+      </c>
+      <c r="AM1" s="7" t="inlineStr">
+        <is>
+          <t>第2日计划</t>
+        </is>
+      </c>
+      <c r="AN1" s="7" t="inlineStr">
+        <is>
+          <t>第3日止损</t>
+        </is>
+      </c>
+      <c r="AO1" s="7" t="inlineStr">
+        <is>
+          <t>第3日止盈</t>
+        </is>
+      </c>
+      <c r="AP1" s="7" t="inlineStr">
+        <is>
+          <t>第3日计划</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="4" t="n">
@@ -1357,7 +1420,7 @@
         </is>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB2" s="4" t="n">
         <v>127.36</v>
@@ -1376,7 +1439,40 @@
       </c>
       <c r="AG2" s="4" t="inlineStr">
         <is>
-          <t>3日计划；跌破127.36止损；上冲152.29先止盈；破MA5/移动止盈128.67减仓</t>
+          <t>1日短线计划；T+1看145.58/止损132.16；T+2看148.45/止损127.98；T+3看152.29/止损128.67</t>
+        </is>
+      </c>
+      <c r="AH2" s="4" t="n">
+        <v>132.16</v>
+      </c>
+      <c r="AI2" s="4" t="n">
+        <v>145.58</v>
+      </c>
+      <c r="AJ2" s="4" t="inlineStr">
+        <is>
+          <t>T+1：冲到145.58先减仓，跌破132.16止损；若高开低走不恋战</t>
+        </is>
+      </c>
+      <c r="AK2" s="4" t="n">
+        <v>127.98</v>
+      </c>
+      <c r="AL2" s="4" t="n">
+        <v>148.45</v>
+      </c>
+      <c r="AM2" s="4" t="inlineStr">
+        <is>
+          <t>T+2：未突破148.45且量能转弱则减仓，跌破127.98退出</t>
+        </is>
+      </c>
+      <c r="AN2" s="4" t="n">
+        <v>128.67</v>
+      </c>
+      <c r="AO2" s="4" t="n">
+        <v>152.29</v>
+      </c>
+      <c r="AP2" s="4" t="inlineStr">
+        <is>
+          <t>T+3：到152.29分批止盈，跌破128.67或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -1466,7 +1562,7 @@
         </is>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB3" s="4" t="n">
         <v>21.87</v>
@@ -1485,7 +1581,40 @@
       </c>
       <c r="AG3" s="4" t="inlineStr">
         <is>
-          <t>3日计划；跌破21.87止损；上冲26.41先止盈；破MA5/移动止盈22.02减仓</t>
+          <t>1日短线计划；T+1看25.06/止损22.70；T+2看25.83/止损22.14；T+3看26.41/止损22.02</t>
+        </is>
+      </c>
+      <c r="AH3" s="4" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="AI3" s="4" t="n">
+        <v>25.06</v>
+      </c>
+      <c r="AJ3" s="4" t="inlineStr">
+        <is>
+          <t>T+1：冲到25.06先减仓，跌破22.70止损；若高开低走不恋战</t>
+        </is>
+      </c>
+      <c r="AK3" s="4" t="n">
+        <v>22.14</v>
+      </c>
+      <c r="AL3" s="4" t="n">
+        <v>25.83</v>
+      </c>
+      <c r="AM3" s="4" t="inlineStr">
+        <is>
+          <t>T+2：未突破25.83且量能转弱则减仓，跌破22.14退出</t>
+        </is>
+      </c>
+      <c r="AN3" s="4" t="n">
+        <v>22.02</v>
+      </c>
+      <c r="AO3" s="4" t="n">
+        <v>26.41</v>
+      </c>
+      <c r="AP3" s="4" t="inlineStr">
+        <is>
+          <t>T+3：到26.41分批止盈，跌破22.02或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -1575,7 +1704,7 @@
         </is>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB4" s="4" t="n">
         <v>66.62</v>
@@ -1594,7 +1723,40 @@
       </c>
       <c r="AG4" s="4" t="inlineStr">
         <is>
-          <t>3日计划；跌破66.62止损；上冲79.90先止盈；破MA5/移动止盈66.62减仓</t>
+          <t>1日短线计划；T+1看76.14/止损69.12；T+2看78.25/止损66.62；T+3看79.90/止损66.62</t>
+        </is>
+      </c>
+      <c r="AH4" s="4" t="n">
+        <v>69.12</v>
+      </c>
+      <c r="AI4" s="4" t="n">
+        <v>76.14</v>
+      </c>
+      <c r="AJ4" s="4" t="inlineStr">
+        <is>
+          <t>T+1：冲到76.14先减仓，跌破69.12止损；若高开低走不恋战</t>
+        </is>
+      </c>
+      <c r="AK4" s="4" t="n">
+        <v>66.62</v>
+      </c>
+      <c r="AL4" s="4" t="n">
+        <v>78.25</v>
+      </c>
+      <c r="AM4" s="4" t="inlineStr">
+        <is>
+          <t>T+2：未突破78.25且量能转弱则减仓，跌破66.62退出</t>
+        </is>
+      </c>
+      <c r="AN4" s="4" t="n">
+        <v>66.62</v>
+      </c>
+      <c r="AO4" s="4" t="n">
+        <v>79.90000000000001</v>
+      </c>
+      <c r="AP4" s="4" t="inlineStr">
+        <is>
+          <t>T+3：到79.90分批止盈，跌破66.62或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1846,7 @@
         </is>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="4" t="n">
         <v>63.96</v>
@@ -1703,7 +1865,40 @@
       </c>
       <c r="AG5" s="4" t="inlineStr">
         <is>
-          <t>3日计划；跌破63.96止损；上冲76.47先止盈；破MA5/移动止盈64.56减仓</t>
+          <t>1日短线计划；T+1看73.10/止损66.36；T+2看74.55/止损64.21；T+3看76.47/止损64.56</t>
+        </is>
+      </c>
+      <c r="AH5" s="4" t="n">
+        <v>66.36</v>
+      </c>
+      <c r="AI5" s="4" t="n">
+        <v>73.09999999999999</v>
+      </c>
+      <c r="AJ5" s="4" t="inlineStr">
+        <is>
+          <t>T+1：冲到73.10先减仓，跌破66.36止损；若高开低走不恋战</t>
+        </is>
+      </c>
+      <c r="AK5" s="4" t="n">
+        <v>64.20999999999999</v>
+      </c>
+      <c r="AL5" s="4" t="n">
+        <v>74.55</v>
+      </c>
+      <c r="AM5" s="4" t="inlineStr">
+        <is>
+          <t>T+2：未突破74.55且量能转弱则减仓，跌破64.21退出</t>
+        </is>
+      </c>
+      <c r="AN5" s="4" t="n">
+        <v>64.56</v>
+      </c>
+      <c r="AO5" s="4" t="n">
+        <v>76.47</v>
+      </c>
+      <c r="AP5" s="4" t="inlineStr">
+        <is>
+          <t>T+3：到76.47分批止盈，跌破64.56或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1988,7 @@
         </is>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB6" s="4" t="n">
         <v>20.04</v>
@@ -1812,7 +2007,40 @@
       </c>
       <c r="AG6" s="4" t="inlineStr">
         <is>
-          <t>3日计划；跌破20.04止损；上冲23.96先止盈；破MA5/移动止盈20.14减仓</t>
+          <t>1日短线计划；T+1看22.91/止损20.80；T+2看23.36/止损20.04；T+3看23.96/止损20.14</t>
+        </is>
+      </c>
+      <c r="AH6" s="4" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="AI6" s="4" t="n">
+        <v>22.91</v>
+      </c>
+      <c r="AJ6" s="4" t="inlineStr">
+        <is>
+          <t>T+1：冲到22.91先减仓，跌破20.80止损；若高开低走不恋战</t>
+        </is>
+      </c>
+      <c r="AK6" s="4" t="n">
+        <v>20.04</v>
+      </c>
+      <c r="AL6" s="4" t="n">
+        <v>23.36</v>
+      </c>
+      <c r="AM6" s="4" t="inlineStr">
+        <is>
+          <t>T+2：未突破23.36且量能转弱则减仓，跌破20.04退出</t>
+        </is>
+      </c>
+      <c r="AN6" s="4" t="n">
+        <v>20.14</v>
+      </c>
+      <c r="AO6" s="4" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AP6" s="4" t="inlineStr">
+        <is>
+          <t>T+3：到23.96分批止盈，跌破20.14或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -1902,7 +2130,7 @@
         </is>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB7" s="4" t="n">
         <v>9.970000000000001</v>
@@ -1921,7 +2149,40 @@
       </c>
       <c r="AG7" s="4" t="inlineStr">
         <is>
-          <t>3日计划；跌破9.97止损；上冲11.92先止盈；破MA5/移动止盈9.97减仓</t>
+          <t>1日短线计划；T+1看11.40/止损10.34；T+2看11.62/止损9.97；T+3看11.92/止损9.97</t>
+        </is>
+      </c>
+      <c r="AH7" s="4" t="n">
+        <v>10.34</v>
+      </c>
+      <c r="AI7" s="4" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="AJ7" s="4" t="inlineStr">
+        <is>
+          <t>T+1：冲到11.40先减仓，跌破10.34止损；若高开低走不恋战</t>
+        </is>
+      </c>
+      <c r="AK7" s="4" t="n">
+        <v>9.970000000000001</v>
+      </c>
+      <c r="AL7" s="4" t="n">
+        <v>11.62</v>
+      </c>
+      <c r="AM7" s="4" t="inlineStr">
+        <is>
+          <t>T+2：未突破11.62且量能转弱则减仓，跌破9.97退出</t>
+        </is>
+      </c>
+      <c r="AN7" s="4" t="n">
+        <v>9.970000000000001</v>
+      </c>
+      <c r="AO7" s="4" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="AP7" s="4" t="inlineStr">
+        <is>
+          <t>T+3：到11.92分批止盈，跌破9.97或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2272,7 @@
         </is>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB8" s="4" t="n">
         <v>46.16</v>
@@ -2030,7 +2291,40 @@
       </c>
       <c r="AG8" s="4" t="inlineStr">
         <is>
-          <t>3日计划；跌破46.16止损；上冲55.23先止盈；破MA5/移动止盈46.16减仓</t>
+          <t>1日短线计划；T+1看52.76/止损47.89；T+2看54.11/止损46.35；T+3看55.23/止损46.16</t>
+        </is>
+      </c>
+      <c r="AH8" s="4" t="n">
+        <v>47.89</v>
+      </c>
+      <c r="AI8" s="4" t="n">
+        <v>52.76</v>
+      </c>
+      <c r="AJ8" s="4" t="inlineStr">
+        <is>
+          <t>T+1：冲到52.76先减仓，跌破47.89止损；若高开低走不恋战</t>
+        </is>
+      </c>
+      <c r="AK8" s="4" t="n">
+        <v>46.35</v>
+      </c>
+      <c r="AL8" s="4" t="n">
+        <v>54.11</v>
+      </c>
+      <c r="AM8" s="4" t="inlineStr">
+        <is>
+          <t>T+2：未突破54.11且量能转弱则减仓，跌破46.35退出</t>
+        </is>
+      </c>
+      <c r="AN8" s="4" t="n">
+        <v>46.16</v>
+      </c>
+      <c r="AO8" s="4" t="n">
+        <v>55.23</v>
+      </c>
+      <c r="AP8" s="4" t="inlineStr">
+        <is>
+          <t>T+3：到55.23分批止盈，跌破46.16或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2414,7 @@
         </is>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB9" s="4" t="n">
         <v>25.9</v>
@@ -2139,7 +2433,40 @@
       </c>
       <c r="AG9" s="4" t="inlineStr">
         <is>
-          <t>3日计划；跌破25.90止损；上冲31.22先止盈；破MA5/移动止盈25.90减仓</t>
+          <t>1日短线计划；T+1看29.65/止损26.88；T+2看30.55/止损25.90；T+3看31.22/止损25.90</t>
+        </is>
+      </c>
+      <c r="AH9" s="4" t="n">
+        <v>26.88</v>
+      </c>
+      <c r="AI9" s="4" t="n">
+        <v>29.65</v>
+      </c>
+      <c r="AJ9" s="4" t="inlineStr">
+        <is>
+          <t>T+1：冲到29.65先减仓，跌破26.88止损；若高开低走不恋战</t>
+        </is>
+      </c>
+      <c r="AK9" s="4" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="AL9" s="4" t="n">
+        <v>30.55</v>
+      </c>
+      <c r="AM9" s="4" t="inlineStr">
+        <is>
+          <t>T+2：未突破30.55且量能转弱则减仓，跌破25.90退出</t>
+        </is>
+      </c>
+      <c r="AN9" s="4" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="AO9" s="4" t="n">
+        <v>31.22</v>
+      </c>
+      <c r="AP9" s="4" t="inlineStr">
+        <is>
+          <t>T+3：到31.22分批止盈，跌破25.90或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2556,7 @@
         </is>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB10" s="4" t="n">
         <v>12.55</v>
@@ -2248,7 +2575,40 @@
       </c>
       <c r="AG10" s="4" t="inlineStr">
         <is>
-          <t>3日计划；跌破12.55止损；上冲15.00先止盈；破MA5/移动止盈12.55减仓</t>
+          <t>1日短线计划；T+1看14.34/止损13.02；T+2看14.62/止损12.55；T+3看15.00/止损12.55</t>
+        </is>
+      </c>
+      <c r="AH10" s="4" t="n">
+        <v>13.02</v>
+      </c>
+      <c r="AI10" s="4" t="n">
+        <v>14.34</v>
+      </c>
+      <c r="AJ10" s="4" t="inlineStr">
+        <is>
+          <t>T+1：冲到14.34先减仓，跌破13.02止损；若高开低走不恋战</t>
+        </is>
+      </c>
+      <c r="AK10" s="4" t="n">
+        <v>12.55</v>
+      </c>
+      <c r="AL10" s="4" t="n">
+        <v>14.62</v>
+      </c>
+      <c r="AM10" s="4" t="inlineStr">
+        <is>
+          <t>T+2：未突破14.62且量能转弱则减仓，跌破12.55退出</t>
+        </is>
+      </c>
+      <c r="AN10" s="4" t="n">
+        <v>12.55</v>
+      </c>
+      <c r="AO10" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="AP10" s="4" t="inlineStr">
+        <is>
+          <t>T+3：到15.00分批止盈，跌破12.55或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2698,7 @@
         </is>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AB11" s="4" t="n">
         <v>166.25</v>
@@ -2357,7 +2717,40 @@
       </c>
       <c r="AG11" s="4" t="inlineStr">
         <is>
-          <t>5日计划；跌破166.25止损；上冲198.78先止盈；破MA5/移动止盈167.08减仓</t>
+          <t>2日短线计划；T+1看190.02/止损172.50；T+2看194.05/止损167.93；T+3看198.78/止损167.08</t>
+        </is>
+      </c>
+      <c r="AH11" s="4" t="n">
+        <v>172.5</v>
+      </c>
+      <c r="AI11" s="4" t="n">
+        <v>190.02</v>
+      </c>
+      <c r="AJ11" s="4" t="inlineStr">
+        <is>
+          <t>T+1：冲到190.02先减仓，跌破172.50止损；若高开低走不恋战</t>
+        </is>
+      </c>
+      <c r="AK11" s="4" t="n">
+        <v>167.93</v>
+      </c>
+      <c r="AL11" s="4" t="n">
+        <v>194.05</v>
+      </c>
+      <c r="AM11" s="4" t="inlineStr">
+        <is>
+          <t>T+2：未突破194.05且量能转弱则减仓，跌破167.93退出</t>
+        </is>
+      </c>
+      <c r="AN11" s="4" t="n">
+        <v>167.08</v>
+      </c>
+      <c r="AO11" s="4" t="n">
+        <v>198.78</v>
+      </c>
+      <c r="AP11" s="4" t="inlineStr">
+        <is>
+          <t>T+3：到198.78分批止盈，跌破167.08或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -2447,7 +2840,7 @@
         </is>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AB12" s="4" t="n">
         <v>35.41</v>
@@ -2466,7 +2859,40 @@
       </c>
       <c r="AG12" s="4" t="inlineStr">
         <is>
-          <t>5日计划；跌破35.41止损；上冲42.34先止盈；破MA5/移动止盈36.04减仓</t>
+          <t>2日短线计划；T+1看40.48/止损36.75；T+2看41.28/止损35.87；T+3看42.34/止损36.04</t>
+        </is>
+      </c>
+      <c r="AH12" s="4" t="n">
+        <v>36.75</v>
+      </c>
+      <c r="AI12" s="4" t="n">
+        <v>40.48</v>
+      </c>
+      <c r="AJ12" s="4" t="inlineStr">
+        <is>
+          <t>T+1：冲到40.48先减仓，跌破36.75止损；若高开低走不恋战</t>
+        </is>
+      </c>
+      <c r="AK12" s="4" t="n">
+        <v>35.87</v>
+      </c>
+      <c r="AL12" s="4" t="n">
+        <v>41.28</v>
+      </c>
+      <c r="AM12" s="4" t="inlineStr">
+        <is>
+          <t>T+2：未突破41.28且量能转弱则减仓，跌破35.87退出</t>
+        </is>
+      </c>
+      <c r="AN12" s="4" t="n">
+        <v>36.04</v>
+      </c>
+      <c r="AO12" s="4" t="n">
+        <v>42.34</v>
+      </c>
+      <c r="AP12" s="4" t="inlineStr">
+        <is>
+          <t>T+3：到42.34分批止盈，跌破36.04或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -2556,7 +2982,7 @@
         </is>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB13" s="4" t="n">
         <v>68.54000000000001</v>
@@ -2575,7 +3001,40 @@
       </c>
       <c r="AG13" s="4" t="inlineStr">
         <is>
-          <t>3日计划；跌破68.54止损；上冲81.95先止盈；破MA5/移动止盈68.54减仓</t>
+          <t>1日短线计划；T+1看78.34/止损71.12；T+2看79.89/止损68.54；T+3看81.95/止损68.54</t>
+        </is>
+      </c>
+      <c r="AH13" s="4" t="n">
+        <v>71.12</v>
+      </c>
+      <c r="AI13" s="4" t="n">
+        <v>78.34</v>
+      </c>
+      <c r="AJ13" s="4" t="inlineStr">
+        <is>
+          <t>T+1：冲到78.34先减仓，跌破71.12止损；若高开低走不恋战</t>
+        </is>
+      </c>
+      <c r="AK13" s="4" t="n">
+        <v>68.54000000000001</v>
+      </c>
+      <c r="AL13" s="4" t="n">
+        <v>79.89</v>
+      </c>
+      <c r="AM13" s="4" t="inlineStr">
+        <is>
+          <t>T+2：未突破79.89且量能转弱则减仓，跌破68.54退出</t>
+        </is>
+      </c>
+      <c r="AN13" s="4" t="n">
+        <v>68.54000000000001</v>
+      </c>
+      <c r="AO13" s="4" t="n">
+        <v>81.95</v>
+      </c>
+      <c r="AP13" s="4" t="inlineStr">
+        <is>
+          <t>T+3：到81.95分批止盈，跌破68.54或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -2665,7 +3124,7 @@
         </is>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB14" s="4" t="n">
         <v>107.52</v>
@@ -2684,7 +3143,40 @@
       </c>
       <c r="AG14" s="4" t="inlineStr">
         <is>
-          <t>3日计划；跌破107.52止损；上冲128.01先止盈；破MA5/移动止盈110.15减仓</t>
+          <t>1日短线计划；T+1看122.49/止损111.36；T+2看124.85/止损109.71；T+3看128.01/止损110.15</t>
+        </is>
+      </c>
+      <c r="AH14" s="4" t="n">
+        <v>111.36</v>
+      </c>
+      <c r="AI14" s="4" t="n">
+        <v>122.49</v>
+      </c>
+      <c r="AJ14" s="4" t="inlineStr">
+        <is>
+          <t>T+1：冲到122.49先减仓，跌破111.36止损；若高开低走不恋战</t>
+        </is>
+      </c>
+      <c r="AK14" s="4" t="n">
+        <v>109.71</v>
+      </c>
+      <c r="AL14" s="4" t="n">
+        <v>124.85</v>
+      </c>
+      <c r="AM14" s="4" t="inlineStr">
+        <is>
+          <t>T+2：未突破124.85且量能转弱则减仓，跌破109.71退出</t>
+        </is>
+      </c>
+      <c r="AN14" s="4" t="n">
+        <v>110.15</v>
+      </c>
+      <c r="AO14" s="4" t="n">
+        <v>128.01</v>
+      </c>
+      <c r="AP14" s="4" t="inlineStr">
+        <is>
+          <t>T+3：到128.01分批止盈，跌破110.15或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -2774,7 +3266,7 @@
         </is>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AB15" s="4" t="n">
         <v>8.449999999999999</v>
@@ -2793,7 +3285,40 @@
       </c>
       <c r="AG15" s="4" t="inlineStr">
         <is>
-          <t>5日计划；跌破8.45止损；上冲10.11先止盈；破MA5/移动止盈8.50减仓</t>
+          <t>2日短线计划；T+1看9.66/止损8.77；T+2看9.85/止损8.45；T+3看10.11/止损8.50</t>
+        </is>
+      </c>
+      <c r="AH15" s="4" t="n">
+        <v>8.77</v>
+      </c>
+      <c r="AI15" s="4" t="n">
+        <v>9.66</v>
+      </c>
+      <c r="AJ15" s="4" t="inlineStr">
+        <is>
+          <t>T+1：冲到9.66先减仓，跌破8.77止损；若高开低走不恋战</t>
+        </is>
+      </c>
+      <c r="AK15" s="4" t="n">
+        <v>8.449999999999999</v>
+      </c>
+      <c r="AL15" s="4" t="n">
+        <v>9.85</v>
+      </c>
+      <c r="AM15" s="4" t="inlineStr">
+        <is>
+          <t>T+2：未突破9.85且量能转弱则减仓，跌破8.45退出</t>
+        </is>
+      </c>
+      <c r="AN15" s="4" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="AO15" s="4" t="n">
+        <v>10.11</v>
+      </c>
+      <c r="AP15" s="4" t="inlineStr">
+        <is>
+          <t>T+3：到10.11分批止盈，跌破8.50或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -2883,7 +3408,7 @@
         </is>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB16" s="4" t="n">
         <v>11.25</v>
@@ -2902,7 +3427,40 @@
       </c>
       <c r="AG16" s="4" t="inlineStr">
         <is>
-          <t>3日计划；跌破11.25止损；上冲13.46先止盈；破MA5/移动止盈11.25减仓</t>
+          <t>1日短线计划；T+1看12.86/止损11.68；T+2看13.12/止损11.25；T+3看13.46/止损11.25</t>
+        </is>
+      </c>
+      <c r="AH16" s="4" t="n">
+        <v>11.68</v>
+      </c>
+      <c r="AI16" s="4" t="n">
+        <v>12.86</v>
+      </c>
+      <c r="AJ16" s="4" t="inlineStr">
+        <is>
+          <t>T+1：冲到12.86先减仓，跌破11.68止损；若高开低走不恋战</t>
+        </is>
+      </c>
+      <c r="AK16" s="4" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="AL16" s="4" t="n">
+        <v>13.12</v>
+      </c>
+      <c r="AM16" s="4" t="inlineStr">
+        <is>
+          <t>T+2：未突破13.12且量能转弱则减仓，跌破11.25退出</t>
+        </is>
+      </c>
+      <c r="AN16" s="4" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="AO16" s="4" t="n">
+        <v>13.46</v>
+      </c>
+      <c r="AP16" s="4" t="inlineStr">
+        <is>
+          <t>T+3：到13.46分批止盈，跌破11.25或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -2992,7 +3550,7 @@
         </is>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AB17" s="4" t="n">
         <v>31.73</v>
@@ -3011,7 +3569,40 @@
       </c>
       <c r="AG17" s="4" t="inlineStr">
         <is>
-          <t>5日计划；跌破31.73止损；上冲37.94先止盈；破MA5/移动止盈32.23减仓</t>
+          <t>2日短线计划；T+1看36.27/止损32.93；T+2看36.99/止损32.07；T+3看37.94/止损32.23</t>
+        </is>
+      </c>
+      <c r="AH17" s="4" t="n">
+        <v>32.93</v>
+      </c>
+      <c r="AI17" s="4" t="n">
+        <v>36.27</v>
+      </c>
+      <c r="AJ17" s="4" t="inlineStr">
+        <is>
+          <t>T+1：冲到36.27先减仓，跌破32.93止损；若高开低走不恋战</t>
+        </is>
+      </c>
+      <c r="AK17" s="4" t="n">
+        <v>32.07</v>
+      </c>
+      <c r="AL17" s="4" t="n">
+        <v>36.99</v>
+      </c>
+      <c r="AM17" s="4" t="inlineStr">
+        <is>
+          <t>T+2：未突破36.99且量能转弱则减仓，跌破32.07退出</t>
+        </is>
+      </c>
+      <c r="AN17" s="4" t="n">
+        <v>32.23</v>
+      </c>
+      <c r="AO17" s="4" t="n">
+        <v>37.94</v>
+      </c>
+      <c r="AP17" s="4" t="inlineStr">
+        <is>
+          <t>T+3：到37.94分批止盈，跌破32.23或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -3101,7 +3692,7 @@
         </is>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AB18" s="4" t="n">
         <v>37.8</v>
@@ -3120,7 +3711,40 @@
       </c>
       <c r="AG18" s="4" t="inlineStr">
         <is>
-          <t>5日计划；跌破37.80止损；上冲45.19先止盈；破MA5/移动止盈38.30减仓</t>
+          <t>2日短线计划；T+1看43.20/止损39.22；T+2看44.05/止损38.11；T+3看45.19/止损38.30</t>
+        </is>
+      </c>
+      <c r="AH18" s="4" t="n">
+        <v>39.22</v>
+      </c>
+      <c r="AI18" s="4" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="AJ18" s="4" t="inlineStr">
+        <is>
+          <t>T+1：冲到43.20先减仓，跌破39.22止损；若高开低走不恋战</t>
+        </is>
+      </c>
+      <c r="AK18" s="4" t="n">
+        <v>38.11</v>
+      </c>
+      <c r="AL18" s="4" t="n">
+        <v>44.05</v>
+      </c>
+      <c r="AM18" s="4" t="inlineStr">
+        <is>
+          <t>T+2：未突破44.05且量能转弱则减仓，跌破38.11退出</t>
+        </is>
+      </c>
+      <c r="AN18" s="4" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="AO18" s="4" t="n">
+        <v>45.19</v>
+      </c>
+      <c r="AP18" s="4" t="inlineStr">
+        <is>
+          <t>T+3：到45.19分批止盈，跌破38.30或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3834,7 @@
         </is>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB19" s="4" t="n">
         <v>43.34</v>
@@ -3229,7 +3853,40 @@
       </c>
       <c r="AG19" s="4" t="inlineStr">
         <is>
-          <t>3日计划；跌破43.34止损；上冲51.82先止盈；破MA5/移动止盈43.34减仓</t>
+          <t>1日短线计划；T+1看49.54/止损44.97；T+2看50.51/止损43.34；T+3看51.82/止损43.34</t>
+        </is>
+      </c>
+      <c r="AH19" s="4" t="n">
+        <v>44.97</v>
+      </c>
+      <c r="AI19" s="4" t="n">
+        <v>49.54</v>
+      </c>
+      <c r="AJ19" s="4" t="inlineStr">
+        <is>
+          <t>T+1：冲到49.54先减仓，跌破44.97止损；若高开低走不恋战</t>
+        </is>
+      </c>
+      <c r="AK19" s="4" t="n">
+        <v>43.34</v>
+      </c>
+      <c r="AL19" s="4" t="n">
+        <v>50.51</v>
+      </c>
+      <c r="AM19" s="4" t="inlineStr">
+        <is>
+          <t>T+2：未突破50.51且量能转弱则减仓，跌破43.34退出</t>
+        </is>
+      </c>
+      <c r="AN19" s="4" t="n">
+        <v>43.34</v>
+      </c>
+      <c r="AO19" s="4" t="n">
+        <v>51.82</v>
+      </c>
+      <c r="AP19" s="4" t="inlineStr">
+        <is>
+          <t>T+3：到51.82分批止盈，跌破43.34或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -3319,7 +3976,7 @@
         </is>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB20" s="4" t="n">
         <v>73.93000000000001</v>
@@ -3338,7 +3995,40 @@
       </c>
       <c r="AG20" s="4" t="inlineStr">
         <is>
-          <t>3日计划；跌破73.93止损；上冲88.39先止盈；破MA5/移动止盈74.37减仓</t>
+          <t>1日短线计划；T+1看84.50/止损76.71；T+2看86.17/止损74.75；T+3看88.39/止损74.37</t>
+        </is>
+      </c>
+      <c r="AH20" s="4" t="n">
+        <v>76.70999999999999</v>
+      </c>
+      <c r="AI20" s="4" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="AJ20" s="4" t="inlineStr">
+        <is>
+          <t>T+1：冲到84.50先减仓，跌破76.71止损；若高开低走不恋战</t>
+        </is>
+      </c>
+      <c r="AK20" s="4" t="n">
+        <v>74.75</v>
+      </c>
+      <c r="AL20" s="4" t="n">
+        <v>86.17</v>
+      </c>
+      <c r="AM20" s="4" t="inlineStr">
+        <is>
+          <t>T+2：未突破86.17且量能转弱则减仓，跌破74.75退出</t>
+        </is>
+      </c>
+      <c r="AN20" s="4" t="n">
+        <v>74.37</v>
+      </c>
+      <c r="AO20" s="4" t="n">
+        <v>88.39</v>
+      </c>
+      <c r="AP20" s="4" t="inlineStr">
+        <is>
+          <t>T+3：到88.39分批止盈，跌破74.37或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -3428,7 +4118,7 @@
         </is>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB21" s="4" t="n">
         <v>27.14</v>
@@ -3447,12 +4137,45 @@
       </c>
       <c r="AG21" s="4" t="inlineStr">
         <is>
-          <t>3日计划；跌破27.14止损；上冲32.45先止盈；破MA5/移动止盈27.16减仓</t>
+          <t>1日短线计划；T+1看31.02/止损28.16；T+2看31.69/止损27.30；T+3看32.45/止损27.16</t>
+        </is>
+      </c>
+      <c r="AH21" s="4" t="n">
+        <v>28.16</v>
+      </c>
+      <c r="AI21" s="4" t="n">
+        <v>31.02</v>
+      </c>
+      <c r="AJ21" s="4" t="inlineStr">
+        <is>
+          <t>T+1：冲到31.02先减仓，跌破28.16止损；若高开低走不恋战</t>
+        </is>
+      </c>
+      <c r="AK21" s="4" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="AL21" s="4" t="n">
+        <v>31.69</v>
+      </c>
+      <c r="AM21" s="4" t="inlineStr">
+        <is>
+          <t>T+2：未突破31.69且量能转弱则减仓，跌破27.30退出</t>
+        </is>
+      </c>
+      <c r="AN21" s="4" t="n">
+        <v>27.16</v>
+      </c>
+      <c r="AO21" s="4" t="n">
+        <v>32.45</v>
+      </c>
+      <c r="AP21" s="4" t="inlineStr">
+        <is>
+          <t>T+3：到32.45分批止盈，跌破27.16或MA5失守退出</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AG21"/>
+  <autoFilter ref="A1:AP21"/>
   <conditionalFormatting sqref="G2:G21">
     <cfRule type="colorScale" priority="1">
       <colorScale>

</xml_diff>